<commit_message>
adición de relaciones entre cuentas de recaudado
</commit_message>
<xml_diff>
--- a/public/Guia/Rec-CuentasConceptos.xlsx
+++ b/public/Guia/Rec-CuentasConceptos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\Guia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2C76AD-C482-4C15-9ED6-868B77BF4B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3783735-DCA2-476B-BA3E-6C878CBC2E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -639,8 +638,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="82" customWidth="1"/>
+    <col min="2" max="2" width="61.42578125" customWidth="1"/>
+    <col min="3" max="3" width="93.140625" customWidth="1"/>
     <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>